<commit_message>
Recalculate tracker release window column from End dates
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YRFgXpWYZpZNdiR4z24WSz
</commit_message>
<xml_diff>
--- a/ManageEngine_Interface_Tracker_v3.xlsx
+++ b/ManageEngine_Interface_Tracker_v3.xlsx
@@ -19,8 +19,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="dd-mmm-yy"/>
+    <numFmt numFmtId="164" formatCode="dd-mmm-yy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -71,13 +71,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="17" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -87,6 +87,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -464,6 +467,7 @@
     <col width="21" customWidth="1" min="8" max="8"/>
     <col width="38" customWidth="1" min="9" max="9"/>
     <col width="25.6640625" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.4" customHeight="1">
@@ -522,6 +526,11 @@
           <t>Milestone</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Release Window</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.4" customHeight="1">
       <c r="A2" t="inlineStr">
@@ -1025,9 +1034,9 @@
           <t>Monitoring alerts and performance events</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>Release 1</t>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>Release 2</t>
         </is>
       </c>
     </row>
@@ -1211,9 +1220,9 @@
           <t>SIEM events and security incident data</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>Release 2</t>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>Release 3</t>
         </is>
       </c>
     </row>
@@ -1257,9 +1266,9 @@
           <t>Managed security operations alerts and events</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>Release 2</t>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>Release 3</t>
         </is>
       </c>
     </row>
@@ -1303,9 +1312,9 @@
           <t>Medical device discovery and monitoring</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>Release 2</t>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>Release 3</t>
         </is>
       </c>
     </row>
@@ -1579,9 +1588,9 @@
           <t>Vendor-managed service integration</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>Release 1</t>
+      <c r="L24" s="3" t="inlineStr">
+        <is>
+          <t>Release 3</t>
         </is>
       </c>
     </row>
@@ -1625,9 +1634,9 @@
           <t>Telecommunications service information</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>Release 2</t>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>Release 3</t>
         </is>
       </c>
     </row>
@@ -1671,9 +1680,9 @@
           <t>Vendor-managed service integration</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>Release 2</t>
+      <c r="L26" s="3" t="inlineStr">
+        <is>
+          <t>Release 3</t>
         </is>
       </c>
     </row>
@@ -1717,9 +1726,9 @@
           <t>Vendor-managed service integration</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>Release 2</t>
+      <c r="L27" s="3" t="inlineStr">
+        <is>
+          <t>Release 3</t>
         </is>
       </c>
     </row>
@@ -2118,6 +2127,11 @@
           <t>Historical Cherwell archive repository</t>
         </is>
       </c>
+      <c r="L36" s="3" t="inlineStr">
+        <is>
+          <t>Release 1</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" s="3" t="inlineStr">
@@ -2195,6 +2209,11 @@
       <c r="E39" s="2" t="n">
         <v>46357</v>
       </c>
+      <c r="L39" s="3" t="inlineStr">
+        <is>
+          <t>Release 1</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" t="inlineStr">
@@ -2216,6 +2235,11 @@
       <c r="E40" s="2" t="n">
         <v>46419</v>
       </c>
+      <c r="L40" s="3" t="inlineStr">
+        <is>
+          <t>Release 2</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" t="inlineStr">
@@ -2231,6 +2255,11 @@
       <c r="E41" s="2" t="n">
         <v>46327</v>
       </c>
+      <c r="L41" s="3" t="inlineStr">
+        <is>
+          <t>Release 1</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" t="inlineStr">
@@ -2252,6 +2281,11 @@
       <c r="E42" s="2" t="n">
         <v>46419</v>
       </c>
+      <c r="L42" s="3" t="inlineStr">
+        <is>
+          <t>Release 2</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" t="inlineStr">
@@ -2266,6 +2300,11 @@
       </c>
       <c r="E43" s="2" t="n">
         <v>46508</v>
+      </c>
+      <c r="L43" s="3" t="inlineStr">
+        <is>
+          <t>Release 3</t>
+        </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1">
@@ -2312,7 +2351,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2344,7 +2383,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="n">
+      <c r="A2" s="9" t="n">
         <v>46323</v>
       </c>
       <c r="B2" s="6" t="inlineStr">
@@ -2364,7 +2403,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="n">
+      <c r="A3" s="9" t="n">
         <v>46323</v>
       </c>
       <c r="B3" s="6" t="inlineStr">
@@ -2384,7 +2423,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n">
+      <c r="A4" s="9" t="n">
         <v>46323</v>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -2404,7 +2443,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n">
+      <c r="A5" s="9" t="n">
         <v>46323</v>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -2424,7 +2463,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n">
+      <c r="A6" s="9" t="n">
         <v>46323</v>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -2444,7 +2483,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="n">
+      <c r="A7" s="9" t="n">
         <v>46323</v>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -2464,7 +2503,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n">
+      <c r="A8" s="9" t="n">
         <v>46323</v>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -2484,7 +2523,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n">
+      <c r="A9" s="9" t="n">
         <v>46323</v>
       </c>
       <c r="B9" s="6" t="inlineStr">
@@ -2504,7 +2543,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n">
+      <c r="A10" s="9" t="n">
         <v>46323</v>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -2524,7 +2563,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n">
+      <c r="A11" s="9" t="n">
         <v>46323</v>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -2544,7 +2583,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n">
+      <c r="A12" s="9" t="n">
         <v>46323</v>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -2563,13 +2602,34 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="9" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Call with Jacinta Undy (SVHA)</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Release Window (column L)</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Header added; every row recalculated from End date: Oct-Dec 26 = Release 1, Jan-Mar 27 = Release 2, Apr-Jun 27 = Release 3, Phase/End TBD = TBD. 14 rows changed: Azure Monitoring (Release 1 -&gt; Release 2); LogRhythm (Release 2 -&gt; Release 3); Seamless SOC (Release 2 -&gt; Release 3); Medigate (Release 2 -&gt; Release 3); NTT (Release 1 -&gt; Release 3); Optus (Release 2 -&gt; Release 3); Cognizant (Release 2 -&gt; Release 3); Accenture (Release 2 -&gt; Release 3); Cherwell (blank -&gt; Release 1); Cherwell Shutdown (blank -&gt; Release 1); LivePro Shutdown (blank -&gt; Release 2); ME SDP Release 1 Go Live (blank -&gt; Release 1); ME SDP Release 2 Go Live (blank -&gt; Release 2); ME SDP Release 3 Go Live (blank -&gt; Release 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>Changed cells on 'Interface Tracker' are highlighted light yellow.</t>
         </is>

</xml_diff>